<commit_message>
NPC Data: Added 50+ new opponent sprites
</commit_message>
<xml_diff>
--- a/Spreadsheets/credits.xlsx
+++ b/Spreadsheets/credits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F92BFBBB-58FC-4020-9CB7-2A89EE1750C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB6CA16-06BD-47AE-BFDD-E4BC47AA0A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="69">
   <si>
     <t>In Battle Trainer Sprites</t>
   </si>
@@ -198,13 +198,68 @@
     <t>https://www.deviantart.com/mid117/art/Pokemon-Sun-and-Moon-Team-Skull-Grunts-Sprite-657950401</t>
   </si>
   <si>
-    <t>XY, USUM, ORAS in battle sprites</t>
-  </si>
-  <si>
-    <t>Kyle-Dove</t>
-  </si>
-  <si>
-    <t>https://www.deviantart.com/kyle-dove/gallery</t>
+    <t>Rogue/Rebel trainer sprites (overworld and in battle)</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/gogoat1/gallery/73439897/sprites-and-characters?page=4</t>
+  </si>
+  <si>
+    <t>gogoat1</t>
+  </si>
+  <si>
+    <t>boonzeet</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/boonzeet/gallery</t>
+  </si>
+  <si>
+    <t>wergen</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/wergan/gallery/101032271/gaole</t>
+  </si>
+  <si>
+    <t>Kyle-Dove / kyledove</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/kyle-dove/gallery
+https://eeveeexpo.com/resources/authors/9232/</t>
+  </si>
+  <si>
+    <t>XY, USUM, ORAS, SWSH overworld sprites</t>
+  </si>
+  <si>
+    <t>XY, USUM, ORAS, SWSH in battle sprites</t>
+  </si>
+  <si>
+    <t>Pokemon sword gloria in battle sprite</t>
+  </si>
+  <si>
+    <t>Pokemon sword gloria overworld sprite</t>
+  </si>
+  <si>
+    <t>wolfang</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/wolfang62/art/Hero-of-Galar-Battler-Sprite-Female-788246849</t>
+  </si>
+  <si>
+    <t>ash sprites</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/pkmntrainerrick/art/Ash-Hgss-Dpp-Style-Sprites-Full-pack-950185285</t>
+  </si>
+  <si>
+    <t>pkmntrainerrick</t>
+  </si>
+  <si>
+    <t>seethingcumbucket</t>
+  </si>
+  <si>
+    <t>https://www.reddit.com/r/PokemonRMXP/comments/mhrxup/pokemon_gen_17_overworld_sprites_download_link/</t>
+  </si>
+  <si>
+    <t>Pokemon overworld sprites</t>
   </si>
 </sst>
 </file>
@@ -593,15 +648,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8449EA-7B8C-4284-BC16-D53892B08179}">
-  <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="51.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44.5546875" customWidth="1"/>
-    <col min="3" max="3" width="109.6640625" customWidth="1"/>
+    <col min="1" max="1" width="51.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.5703125" customWidth="1"/>
+    <col min="3" max="3" width="109.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -612,7 +667,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -623,7 +678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -634,7 +689,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -645,7 +700,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>11</v>
       </c>
@@ -653,7 +708,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>12</v>
       </c>
@@ -661,7 +716,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>13</v>
       </c>
@@ -669,7 +724,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -680,7 +735,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -691,7 +746,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -702,7 +757,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -713,7 +768,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -724,7 +779,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -735,7 +790,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -746,7 +801,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="273.60000000000002" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="300" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -757,48 +812,114 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B21" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" t="s">
         <v>49</v>
       </c>
-      <c r="C16" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>39</v>
-      </c>
-      <c r="B17" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>44</v>
-      </c>
-      <c r="B19" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" t="s">
-        <v>47</v>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>60</v>
+      </c>
+      <c r="B22" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" t="s">
+        <v>66</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -807,7 +928,7 @@
     <hyperlink ref="B3" r:id="rId2" display="https://www.reddit.com/user/New_Personality_9208/" xr:uid="{B6FC823D-A351-4968-90C5-AB0A9D22DCC7}"/>
     <hyperlink ref="B10" r:id="rId3" display="https://www.deviantart.com/thecubberx/gallery" xr:uid="{1CE16580-A4E8-4E2A-8B7A-6EEC4BA2FD45}"/>
     <hyperlink ref="B14" r:id="rId4" display="https://www.deviantart.com/aurumdeluxe" xr:uid="{DF54BD18-078B-4049-BEBB-106BDA490062}"/>
-    <hyperlink ref="B18" r:id="rId5" display="https://www.deviantart.com/diegowt/gallery" xr:uid="{5595E6A6-D3C6-401E-81D5-305B7CA40024}"/>
+    <hyperlink ref="B19" r:id="rId5" display="https://www.deviantart.com/diegowt/gallery" xr:uid="{5595E6A6-D3C6-401E-81D5-305B7CA40024}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
NPC Data: Fixed sprite name issues and missing images
</commit_message>
<xml_diff>
--- a/Spreadsheets/credits.xlsx
+++ b/Spreadsheets/credits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDB6CA16-06BD-47AE-BFDD-E4BC47AA0A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A98F340E-87D9-4213-BEF7-0BEB57C454A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
+    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="17145" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="72">
   <si>
     <t>In Battle Trainer Sprites</t>
   </si>
@@ -260,6 +260,15 @@
   </si>
   <si>
     <t>Pokemon overworld sprites</t>
+  </si>
+  <si>
+    <t>Kindler Sprite</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/brawlzilla/gallery?page=5</t>
+  </si>
+  <si>
+    <t>Brawlzilla</t>
   </si>
 </sst>
 </file>
@@ -648,7 +657,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8449EA-7B8C-4284-BC16-D53892B08179}">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51.140625" bestFit="1" customWidth="1"/>
@@ -920,6 +929,17 @@
       </c>
       <c r="C25" s="1" t="s">
         <v>67</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>